<commit_message>
Add a Telski open-positions snapshot alongside the classified analysis
Captured all 36 open positions from the Telluride Ski and Golf job board on August 2, 2026, classified to the same SOC major groups as the newspaper ads. 26 are seasonal against 8 year round. The board publishes no pay figures, so this contributes position counts and the seasonal split rather than wages.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Housing Study/Job Market/Telluride Times print help-wanted with pay.xlsx
+++ b/assets/Housing Study/Job Market/Telluride Times print help-wanted with pay.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advertised pay" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every ad" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and limits" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Telski openings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every ad'!$A$4:$H$176</definedName>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +71,11 @@
       <b val="1"/>
       <color rgb="00B98A2F"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001D5C63"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -110,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +158,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7336,4 +7343,1180 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Telluride Ski and Golf, all open positions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>A single-day snapshot taken from the company job board on August 2, 2026. This is one employer, not the whole market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Open positions</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Year round</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>BLS SOC major group</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Open positions</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Other or not stated</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>49-0000 Installation, Maintenance, and Repair</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>43-0000 Office and Administrative Support</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>41-0000 Sales and Related</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>15-0000 Computer and Mathematical</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>33-0000 Protective Service</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>53-0000 Transportation and Material Moving</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Position title</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Employment type</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>BLS SOC major group</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Administrative Coordinator</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Reception</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>43-0000 Office and Administrative Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Allred's AM Winter Sous Chef</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Allred's Restaurant</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Bon Vivant Operations Manager</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Bon Vivant</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Children's Group Ski Instructor</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Children's Instruction</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Children's Ski &amp; Snowboard School, Rental Technician Supervisor</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Children's Ski &amp; Snowboard School, Indoor Attendant</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Clubhouse Bartender</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Clubhouse</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Golf and Members' Club</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Clubhouse Cook</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Clubhouse</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Golf and Members' Club</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Fully Certified Ski Lesson Instructor</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Other or not stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Inn at Lost Creek Front Office Manager</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Inn at Lost Creek</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Inn at Lost Creek</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Lift Operator I (Winter)</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Lift Operations</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Outside Services Attendant</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Outside Services</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Golf and Members' Club</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Peaks Resort &amp; Spa Cosmetologist</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Peaks Spa</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Spa at The Peaks Resort</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Peaks Resort &amp; Spa Massage Therapist</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Peaks Spa</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Spa at The Peaks Resort</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Private Lessons Supervisor</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Retail Sales Associate - Sunshine / Guest Service Store</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Retail Warehouse Associate/Driver</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>41-0000 Sales and Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Senior Systems Administrator</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Information Systems</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>15-0000 Computer and Mathematical</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Ski Cub Instructor</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Ski School</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Other or not stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Ski Patrol Manager - Training</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Ski Patrol</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>33-0000 Protective Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Ski Valet Attendant</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Slopeside Lockers</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Resort Services</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Snowmaker</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Snowmaking</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>49-0000 Installation, Maintenance, and Repair</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Snowmaking Foreman</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Snowmaking</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Snowmaking Technician</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Snowmaking</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>49-0000 Installation, Maintenance, and Repair</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Spa Concierge</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Peaks Spa</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Spa at The Peaks Resort</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Telluride Sports Cimarron Store Manager</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Telluride Sports Gondola Plaza Store Manager</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Telluride Sports Peaks Store Manager</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>11-0000 Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern Backwaiter</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Other or not stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern Bartender</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern Host</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern Server</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Tomboy Tavern</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>35-0000 Food Preparation and Serving Related</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Trail Safety Team Member</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Trail Safety</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Other or not stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Vehicle Mechanic II</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Vehicle Maintenance</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>49-0000 Installation, Maintenance, and Repair</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Warehouse &amp; Delivery Attendant</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>F &amp; B Admin</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Food and Beverage</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Year Round</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>39-0000 Personal Care and Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Zipline Driver / First Responder</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Zipline Adventures</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Zipline Adventures</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Seasonal</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>53-0000 Transportation and Material Moving</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>